<commit_message>
Más documentos para pruebas
</commit_message>
<xml_diff>
--- a/gemini-1.5-flash-8b.xlsx
+++ b/gemini-1.5-flash-8b.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AG19"/>
+  <dimension ref="A1:AG39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3548,6 +3548,3306 @@
         </is>
       </c>
       <c r="AG19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>2024-1-EderSands-Report.pdf</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>gemini-1.5-flash-8b</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>1915</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Ondar Fishing Company Limited</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>1 fatality</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>North Atlantic</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>Wind westerly at 8kts; 1m seas; dark, with good visibility; estimated sea temperature 14.8°C.</t>
+        </is>
+      </c>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>Shooting fishing gear</t>
+        </is>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T20" t="inlineStr">
+        <is>
+          <t>Yes, the skipper used astern power to stop the vessel and sounded the crew alarm and whistle.</t>
+        </is>
+      </c>
+      <c r="U20" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="V20" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="W20" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="X20" t="inlineStr">
+        <is>
+          <t>1915</t>
+        </is>
+      </c>
+      <c r="Y20" t="inlineStr">
+        <is>
+          <t>20 crew: a Spanish master, mate, chief engineer and bosun and 16 Indonesian nationals.</t>
+        </is>
+      </c>
+      <c r="Z20" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AA20" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AB20" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AC20" t="inlineStr">
+        <is>
+          <t>good visibility</t>
+        </is>
+      </c>
+      <c r="AD20" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AE20" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AF20" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AG20" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>2024-1-EderSands-Report.pdf</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>gemini-1.5-flash-8b</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>About 1915</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Ondar Fishing Company Limited</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>1 fatality</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>North Atlantic</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>Wind westerly at 8kts; 1m seas; dark, with good visibility; estimated sea temperature 14.8°C.</t>
+        </is>
+      </c>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>Shooting fishing gear.</t>
+        </is>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>The text states the crew threw "port and starboard lifebuoys with their smoke and light floats overboard, along with one of the vessel’s foam abandonment lifejackets."</t>
+        </is>
+      </c>
+      <c r="T21" t="inlineStr">
+        <is>
+          <t>Yes, at about 1915, the deckhand shouted to stop the vessel and call the bosun, and the skipper used astern power to stop the vessel and sounded the crew alarm and whistle.  Later, at about 1935, the skipper made "Mayday" calls and activated the DSC alarm.</t>
+        </is>
+      </c>
+      <c r="U21" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="V21" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="W21" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="X21" t="inlineStr">
+        <is>
+          <t>1915</t>
+        </is>
+      </c>
+      <c r="Y21" t="inlineStr">
+        <is>
+          <t>20 crew: a Spanish master, mate, chief engineer and bosun and 16 Indonesian nationals</t>
+        </is>
+      </c>
+      <c r="Z21" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AA21" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AB21" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AC21" t="inlineStr">
+        <is>
+          <t>dark, with good visibility</t>
+        </is>
+      </c>
+      <c r="AD21" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AE21" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AF21" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AG21" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>2023-2-HarrietJ-Report.pdf</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>gemini-1.5-flash-8b</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>0736</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Privately owned</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>West</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>5.4kts</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>1997</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>North Sea</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>Long 1.2m northerly swell; air temperature 12°C; wind south-westerly force 3; sea temperature approximately 15°C</t>
+        </is>
+      </c>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>Shooting the fishing gear.</t>
+        </is>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S22" t="inlineStr">
+        <is>
+          <t>The PFD and PLB were both in the wheelhouse.</t>
+        </is>
+      </c>
+      <c r="T22" t="inlineStr">
+        <is>
+          <t>Yes, a "Mayday Relay" was broadcast.</t>
+        </is>
+      </c>
+      <c r="U22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="V22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="W22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="X22" t="inlineStr">
+        <is>
+          <t>0736</t>
+        </is>
+      </c>
+      <c r="Y22" t="inlineStr">
+        <is>
+          <t>1, the skipper</t>
+        </is>
+      </c>
+      <c r="Z22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AA22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AB22" t="inlineStr">
+        <is>
+          <t>0.5 nautical miles</t>
+        </is>
+      </c>
+      <c r="AC22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AD22" t="inlineStr">
+        <is>
+          <t>Yes, the vessel's speed dipped.</t>
+        </is>
+      </c>
+      <c r="AE22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AF22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AG22" t="inlineStr">
+        <is>
+          <t>0.9nm</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>2023-1-EmmaLouise-Report.pdf</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>gemini-1.5-flash-8b</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>About 1000 on 12 January 2022</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>William Traynor</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>The men were sitting in the cockpit with its canopy closed, each drank a beer.  The alcohol stove had not been used.</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>1996</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>Yes, 2 fatalities</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>Yes, moored and engine running</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>River Hamble</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>Light northerly wind; drizzle; 10°C</t>
+        </is>
+      </c>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>Started the boat’s engine, switched on a portable electric radiator, the cockpit lights, navigation lights and the entertainment radio. They then sat in the cockpit with its canopy closed and each drank a beer.</t>
+        </is>
+      </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>Beer</t>
+        </is>
+      </c>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T23" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="U23" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="V23" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="W23" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="X23" t="inlineStr">
+        <is>
+          <t>early evening</t>
+        </is>
+      </c>
+      <c r="Y23" t="inlineStr">
+        <is>
+          <t>2 men; Emma Louise's owner, William Traynor, and his brother-in-law, Martin Steventon</t>
+        </is>
+      </c>
+      <c r="Z23" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AA23" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AB23" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AC23" t="inlineStr">
+        <is>
+          <t>Light northerly wind; drizzle</t>
+        </is>
+      </c>
+      <c r="AD23" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AE23" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AF23" t="inlineStr">
+        <is>
+          <t>160kg</t>
+        </is>
+      </c>
+      <c r="AG23" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>2023-1-EmmaLouise-Report.pdf</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>gemini-1.5-flash-8b</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Early evening on 11 January 2022</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>William Traynor</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Not applicable; the vessel was moored.</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Yes, the men were sitting in the cockpit, drinking beer.</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>1996</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>Yes, 2 fatalities</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>Yes, the vessel was moored.</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>No notable mechanical failures were mentioned before the incident; however, the exhaust system was modified during the boat's life.</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>River Hamble</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>Light northerly wind; drizzle; 10°C.</t>
+        </is>
+      </c>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>The owner called his wife, they boarded the boat, secured the canopy, and switched on the portable electric radiator.  The men sat in the cockpit, each drank a beer.</t>
+        </is>
+      </c>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>Half a bottle of beer.</t>
+        </is>
+      </c>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S24" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T24" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="U24" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="V24" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="W24" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="X24" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Y24" t="inlineStr">
+        <is>
+          <t>2 men: William Traynor and Martin Steventon</t>
+        </is>
+      </c>
+      <c r="Z24" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AA24" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AB24" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AC24" t="inlineStr">
+        <is>
+          <t>Light northerly wind; drizzle</t>
+        </is>
+      </c>
+      <c r="AD24" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AE24" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AF24" t="inlineStr">
+        <is>
+          <t>160kg</t>
+        </is>
+      </c>
+      <c r="AG24" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>2022-14-ReulAChuain.pdf</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>gemini-1.5-flash-8b</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>1900</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Privately owned</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Mallaig, Scotland</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>6.5 kts</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>1959</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>1 fatality</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>Sound of Rùm</t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>good with a force 4 south-westerly wind, then veered to the north and increased to a force 6, creating a short steep swell</t>
+        </is>
+      </c>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>sorting the last of the prawns and stowing the boxes in the fish hold</t>
+        </is>
+      </c>
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>Mallaig ALB</t>
+        </is>
+      </c>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>Foredeck of Reul A Chuain</t>
+        </is>
+      </c>
+      <c r="T25" t="inlineStr">
+        <is>
+          <t>Yes, the junior deckhand made a distress call on very high frequency channel 16.</t>
+        </is>
+      </c>
+      <c r="U25" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="V25" t="inlineStr">
+        <is>
+          <t>No, the nets were not routinely lashed at the end of the day's fishing, allowing them to slip overboard.</t>
+        </is>
+      </c>
+      <c r="W25" t="inlineStr">
+        <is>
+          <t>No, the crew had not practised man overboard recovery and were unfamiliar with the vessel's man overboard recovery equipment.</t>
+        </is>
+      </c>
+      <c r="X25" t="inlineStr">
+        <is>
+          <t>24 June 2021</t>
+        </is>
+      </c>
+      <c r="Y25" t="inlineStr">
+        <is>
+          <t>Three crew members; skipper, senior deckhand, and junior deckhand</t>
+        </is>
+      </c>
+      <c r="Z25" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AA25" t="inlineStr">
+        <is>
+          <t>0 hours 45 minutes</t>
+        </is>
+      </c>
+      <c r="AB25" t="inlineStr">
+        <is>
+          <t>Yes; Ronja Harvester (distance not provided)</t>
+        </is>
+      </c>
+      <c r="AC25" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AD25" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AE25" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AF25" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AG25" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>2022-14-ReulAChuain.pdf</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>gemini-1.5-flash-8b</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>1900</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Privately owned</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Mallaig, Scotland</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>6.5 kts</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>1959</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>1 fatality</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>Sound of Rùm</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>good with a force 4 south-westerly wind; veered to the north and increased to a force 6, creating a short steep swell</t>
+        </is>
+      </c>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>The crew member was recovering a net that had slipped overboard.</t>
+        </is>
+      </c>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>Mallaig ALB</t>
+        </is>
+      </c>
+      <c r="S26" t="inlineStr">
+        <is>
+          <t>Foredeck of Reul A Chuain</t>
+        </is>
+      </c>
+      <c r="T26" t="inlineStr">
+        <is>
+          <t>Yes, a distress call was made on VHF channel 16 at about 1906.</t>
+        </is>
+      </c>
+      <c r="U26" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="V26" t="inlineStr">
+        <is>
+          <t>The cargo of boxed prawns was being sorted and stowed in the fish hold.</t>
+        </is>
+      </c>
+      <c r="W26" t="inlineStr">
+        <is>
+          <t>No, the crew had not practiced man overboard recovery drills and were unfamiliar with the vessel's man overboard recovery equipment.</t>
+        </is>
+      </c>
+      <c r="X26" t="inlineStr">
+        <is>
+          <t>24 June 2021</t>
+        </is>
+      </c>
+      <c r="Y26" t="inlineStr">
+        <is>
+          <t>Three crew members; a skipper and two deckhands.</t>
+        </is>
+      </c>
+      <c r="Z26" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AA26" t="inlineStr">
+        <is>
+          <t>1 hour and 5 minutes</t>
+        </is>
+      </c>
+      <c r="AB26" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AC26" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AD26" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AE26" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AF26" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AG26" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>2022-11-Goodway-Report.pdf</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>gemini-1.5-flash-8b</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>1340 on 16 October 2021</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Joe Masson</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Cairnbulg Briggs reef, north-east of Cairnbulg Point</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>2004</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>One presumed fatality</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>North Sea</t>
+        </is>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>Wind direction was variable but mainly westerly force 2 to 3, slight sea, low north-westerly swell, sea temperature 12°C, visibility good.</t>
+        </is>
+      </c>
+      <c r="P27" t="inlineStr">
+        <is>
+          <t>Fishing alone, near where his vessel was found, anchored to a fleet of creels on the seabed.</t>
+        </is>
+      </c>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S27" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T27" t="inlineStr">
+        <is>
+          <t>No VHF, DSC or AIS distress alert was received from Goodway.</t>
+        </is>
+      </c>
+      <c r="U27" t="inlineStr">
+        <is>
+          <t>Yes, the owner of Goodway had been previously inspected by the MCA.  Previous inspections had revealed numerous deficiencies.  The skipper of the creel fishing vessel Saint Peter died after becoming caught in his fishing gear and was dragged overboard.  The skipper of the creel vessel Harriet J also died after becoming entangled in the fishing gear.</t>
+        </is>
+      </c>
+      <c r="V27" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="W27" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="X27" t="inlineStr">
+        <is>
+          <t>1340</t>
+        </is>
+      </c>
+      <c r="Y27" t="inlineStr">
+        <is>
+          <t>One, the owner</t>
+        </is>
+      </c>
+      <c r="Z27" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AA27" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AB27" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AC27" t="inlineStr">
+        <is>
+          <t>visibility good.</t>
+        </is>
+      </c>
+      <c r="AD27" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AE27" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AF27" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AG27" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>2022-11-Goodway-Report.pdf</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>gemini-1.5-flash-8b</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>1340 on 16 October 2021</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Joe Masson</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Cairnbulg Briggs reef, north-east of Cairnbulg Point</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>2004</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>Yes, one presumed fatality.</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>No, the vessel was operating with a single person on board.</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>North Sea</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>Wind force 2 to 3, slight sea, low swell, sea temperature 12°C, visibility good.</t>
+        </is>
+      </c>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>Fishing alone, near his vessel, anchored to a fleet of creels on the seabed.</t>
+        </is>
+      </c>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>-.</t>
+        </is>
+      </c>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>-.</t>
+        </is>
+      </c>
+      <c r="S28" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T28" t="inlineStr">
+        <is>
+          <t>No VHF, DSC or AIS distress alert was received from Goodway.</t>
+        </is>
+      </c>
+      <c r="U28" t="inlineStr">
+        <is>
+          <t>Yes, the skipper of the creel fishing vessel Saint Peter died after he became caught in his fishing gear and was dragged overboard, and the skipper of the creel vessel Harriet J died after he became entangled in the fishing gear.</t>
+        </is>
+      </c>
+      <c r="V28" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="W28" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="X28" t="inlineStr">
+        <is>
+          <t>1340</t>
+        </is>
+      </c>
+      <c r="Y28" t="inlineStr">
+        <is>
+          <t>1, the owner</t>
+        </is>
+      </c>
+      <c r="Z28" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AA28" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AB28" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AC28" t="inlineStr">
+        <is>
+          <t>visibility good.</t>
+        </is>
+      </c>
+      <c r="AD28" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AE28" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AF28" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AG28" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>2022-10-Bella-Report.pdf</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>gemini-1.5-flash-8b</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>About 1506 on 6 July 2021</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Geosight Limited</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>North-west</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>About 5 knots</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>2001</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>approaches to Lynmouth</t>
+        </is>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>Wind north-westerly force 3; wave height 0.5m-1.0m</t>
+        </is>
+      </c>
+      <c r="P29" t="inlineStr">
+        <is>
+          <t>lowered the multibeam echo sounder gantry from its stowed position into the sea.</t>
+        </is>
+      </c>
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>rigid inflatable boats (RIB)</t>
+        </is>
+      </c>
+      <c r="S29" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T29" t="inlineStr">
+        <is>
+          <t>Yes, the crew member made a "Mayday!" call using the hand-held VHF radio, which was not answered, and then used a mobile phone to report the emergency to the supervisor ashore. They also called 999 to notify the coastguard.</t>
+        </is>
+      </c>
+      <c r="U29" t="inlineStr">
+        <is>
+          <t>Yes, in 2005, the MAIB investigated the hull failure of the RIB "Big Yellow."</t>
+        </is>
+      </c>
+      <c r="V29" t="inlineStr">
+        <is>
+          <t>No cargo information was mentioned.</t>
+        </is>
+      </c>
+      <c r="W29" t="inlineStr">
+        <is>
+          <t>The skipper held a seafarer's medical certificate and an RYA accredited sea survival course. The crew member had been briefed by the skipper.  The shore supervisor had an RYA Level 2 Powerboat Handling (RYA PBL2) qualification, but without commercial endorsement.</t>
+        </is>
+      </c>
+      <c r="X29" t="inlineStr">
+        <is>
+          <t>1506</t>
+        </is>
+      </c>
+      <c r="Y29" t="inlineStr">
+        <is>
+          <t>2 crew: skipper and crew member</t>
+        </is>
+      </c>
+      <c r="Z29" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AA29" t="inlineStr">
+        <is>
+          <t>0 hours 20 minutes</t>
+        </is>
+      </c>
+      <c r="AB29" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AC29" t="inlineStr">
+        <is>
+          <t>Daylight</t>
+        </is>
+      </c>
+      <c r="AD29" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AE29" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AF29" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AG29" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>2022-10-Bella-Report.pdf</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>gemini-1.5-flash-8b</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>About 1506 on 6 July 2021</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Geosight Limited</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>North-west</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>About 5 knots</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>2001</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>approaches to Lynmouth</t>
+        </is>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>Wind north-westerly force 3; wave height 0.5m-1.0m</t>
+        </is>
+      </c>
+      <c r="P30" t="inlineStr">
+        <is>
+          <t>lowered the multibeam echo sounder (MBES) gantry from its stowed position into the sea</t>
+        </is>
+      </c>
+      <c r="Q30" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R30" t="inlineStr">
+        <is>
+          <t>rigid inflatable boats (RIB)</t>
+        </is>
+      </c>
+      <c r="S30" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T30" t="inlineStr">
+        <is>
+          <t>Yes, the crew member made a "Mayday!" call using a hand-held VHF radio, and then used a mobile phone to report the emergency to the supervisor ashore, and then called 999 to notify the coastguard.</t>
+        </is>
+      </c>
+      <c r="U30" t="inlineStr">
+        <is>
+          <t>Yes, the MAIB investigated the hull failure of the RIB Big Yellow in 2005.</t>
+        </is>
+      </c>
+      <c r="V30" t="inlineStr">
+        <is>
+          <t>No cargo was mentioned.</t>
+        </is>
+      </c>
+      <c r="W30" t="inlineStr">
+        <is>
+          <t>The skipper had completed an RYA accredited sea survival course, and the crew member had been briefed by the skipper.  However, the shore supervisor did not have commercial endorsement, the crew member did not hold a valid seafarers' medical certificate, and the skipper only held lesser qualifications than required by The Workboat Code.</t>
+        </is>
+      </c>
+      <c r="X30" t="inlineStr">
+        <is>
+          <t>1506</t>
+        </is>
+      </c>
+      <c r="Y30" t="inlineStr">
+        <is>
+          <t>2 crew; skipper and crew member</t>
+        </is>
+      </c>
+      <c r="Z30" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AA30" t="inlineStr">
+        <is>
+          <t>0 hours 20 minutes</t>
+        </is>
+      </c>
+      <c r="AB30" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AC30" t="inlineStr">
+        <is>
+          <t>Daylight</t>
+        </is>
+      </c>
+      <c r="AD30" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AE30" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AF30" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AG30" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>2022-6-SaintPeter-Report.pdf</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>gemini-1.5-flash-8b</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>0830</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Privately owned</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Cove, Scotland (intended)</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>1993</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>North Sea</t>
+        </is>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P31" t="inlineStr">
+        <is>
+          <t>shooting creels</t>
+        </is>
+      </c>
+      <c r="Q31" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S31" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T31" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+      <c r="U31" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="V31" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="W31" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="X31" t="inlineStr">
+        <is>
+          <t>0830</t>
+        </is>
+      </c>
+      <c r="Y31" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Z31" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AA31" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AB31" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AC31" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AD31" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AE31" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AF31" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AG31" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>2022-6-SaintPeter-Report.pdf</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>gemini-1.5-flash-8b</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>0830</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Privately owned</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Cove, Scotland (intended)</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>1993</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>North Sea</t>
+        </is>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>shooting creels</t>
+        </is>
+      </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S32" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T32" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+      <c r="U32" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="V32" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="W32" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="X32" t="inlineStr">
+        <is>
+          <t>0830</t>
+        </is>
+      </c>
+      <c r="Y32" t="inlineStr">
+        <is>
+          <t>Owner/skipper (the skipper)</t>
+        </is>
+      </c>
+      <c r="Z32" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AA32" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AB32" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AC32" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AD32" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AE32" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AF32" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AG32" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>2021-14-Achieve-Talis-Report.pdf</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>gemini-1.5-flash-8b</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>1541</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>WeShips Denizcilik ve Ticaret A.Ş.</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Tynemouth</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>The deckhand was boxing up the day's catch on Achieve.</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>The text states that Talis continued on passage at reduced speed, but it doesn't give a speed for Achieve.</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>1997</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>Overcast, poor visibility in patchy fog.  Light southerly wind.</t>
+        </is>
+      </c>
+      <c r="P33" t="inlineStr">
+        <is>
+          <t>Talis’s chief officer (C/O) was on the bridge, carrying out administrative navigation duties at the chart table and the bridge computer. The AB was on the port side.</t>
+        </is>
+      </c>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>Tynemouth RNLI all-weather lifeboat (ALB)</t>
+        </is>
+      </c>
+      <c r="S33" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T33" t="inlineStr">
+        <is>
+          <t>Achieve's skipper called Humber Coastguard on VHF radio channel 16 and advised them he had been in a collision and was taking on water. The VHF call was overheard by the Talis bridge team.</t>
+        </is>
+      </c>
+      <c r="U33" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="V33" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="W33" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="X33" t="inlineStr">
+        <is>
+          <t>1600</t>
+        </is>
+      </c>
+      <c r="Y33" t="inlineStr">
+        <is>
+          <t>A skipper and a deckhand were onboard Achieve. Talis's chief officer (C/O) and duty able-bodied seaman (AB) were onboard Talis.</t>
+        </is>
+      </c>
+      <c r="Z33" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AA33" t="inlineStr">
+        <is>
+          <t>0 hours 5 minutes</t>
+        </is>
+      </c>
+      <c r="AB33" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AC33" t="inlineStr">
+        <is>
+          <t>overcast with fog patches.</t>
+        </is>
+      </c>
+      <c r="AD33" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AE33" t="inlineStr">
+        <is>
+          <t>14 hours.</t>
+        </is>
+      </c>
+      <c r="AF33" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AG33" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>2021-14-Achieve-Talis-Report.pdf</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>gemini-1.5-flash-8b</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>1541</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>WeShips Denizcilik ve Ticaret A.Ş.</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Terneuzen, Netherlands</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>1997</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>Overcast, poor visibility in patchy fog, light southerly wind.</t>
+        </is>
+      </c>
+      <c r="P34" t="inlineStr">
+        <is>
+          <t>Talis’s chief officer (C/O) arrived on the bridge to start his watch, contacted the duty able-bodied seaman (AB) to come to the bridge, the AB arrived shortly after 1505, at 1515 the master left the bridge and went to his cabin, and the C/O carried out administrative navigation duties at the chart table and the bridge computer.  At about 1538, the C/O looked at the starboard radar and observed a target at less than 1nm range. The C/O reduced the radar range scale to 3nm.</t>
+        </is>
+      </c>
+      <c r="Q34" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R34" t="inlineStr">
+        <is>
+          <t>Tynemouth RNLI all-weather lifeboat (ALB)</t>
+        </is>
+      </c>
+      <c r="S34" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T34" t="inlineStr">
+        <is>
+          <t>Achieve's skipper called Humber Coastguard on VHF channel 16.</t>
+        </is>
+      </c>
+      <c r="U34" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="V34" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="W34" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="X34" t="inlineStr">
+        <is>
+          <t>1600</t>
+        </is>
+      </c>
+      <c r="Y34" t="inlineStr">
+        <is>
+          <t>A skipper and a deckhand were onboard Achieve; Talis's chief officer (C/O) and an able-bodied seaman (AB) were onboard Talis.</t>
+        </is>
+      </c>
+      <c r="Z34" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AA34" t="inlineStr">
+        <is>
+          <t>0 hours 15 minutes</t>
+        </is>
+      </c>
+      <c r="AB34" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AC34" t="inlineStr">
+        <is>
+          <t>overcast with fog patches</t>
+        </is>
+      </c>
+      <c r="AD34" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AE34" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AF34" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AG34" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>2021-10-Globetrotter-Report.pdf</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>gemini-1.5-flash-8b</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>0724</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>The owner of Globetrotter</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>To the fishing grounds, to the south of the Lune wind farm.</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>One</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>On passage</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>Steering problems immediately after grounding.</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>Yes, a "Mayday" call was sent out on VHF channel 16 at approximately 0742.</t>
+        </is>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>off the coast of Fleetwood, England</t>
+        </is>
+      </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>fine and clear, easterly Beaufort force 3 to 4, ebbing tide in a south-westerly direction at a rate of about 0.6 knot, sea water temperature was 15.3°C</t>
+        </is>
+      </c>
+      <c r="P35" t="inlineStr">
+        <is>
+          <t>Those on board Fivebuoys were rigging their fishing lines.</t>
+        </is>
+      </c>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R35" t="inlineStr">
+        <is>
+          <t>RNLI inshore lifeboat and Fleetwood’s all-weather lifeboat</t>
+        </is>
+      </c>
+      <c r="S35" t="inlineStr">
+        <is>
+          <t>A pack of parachute flares, two lifebuoys, and a number of buoyancy aids were stowed in the forward cabin. A new automatic-inflation lifejacket was hanging on a hook inside the wheelhouse door. The lifebuoys were stowed in a holder on top of the wheelhouse roof, along with assorted ropes and a grapnel type anchor.  The anchor chain was connected to the foredeck by a length of synthetic rope.</t>
+        </is>
+      </c>
+      <c r="T35" t="inlineStr">
+        <is>
+          <t>Yes.  Globetrotter's owner contacted Fivebuoys' skipper by mobile telephone at 0724, and then, at 0742, used a hand-held VHF radio to broadcast a "Mayday" on VHF channel 16 to Holyhead Coastguard.  He also called Fivebuoys' skipper on his mobile phone again at 0747.</t>
+        </is>
+      </c>
+      <c r="U35" t="inlineStr">
+        <is>
+          <t>Globetrotter's history could not be traced prior to January 2019.</t>
+        </is>
+      </c>
+      <c r="V35" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="W35" t="inlineStr">
+        <is>
+          <t>No.  Globetrotter's owner and his friend had no formal maritime qualifications and had not completed any safety courses.</t>
+        </is>
+      </c>
+      <c r="X35" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Y35" t="inlineStr">
+        <is>
+          <t>Three men: the owner, his son, and his friend.</t>
+        </is>
+      </c>
+      <c r="Z35" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AA35" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AB35" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AC35" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AD35" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AE35" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AF35" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AG35" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>2021-06-BeinnNaCaillich.pdf</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>gemini-1.5-flash-8b</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>1510</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Marine Harvest (Scotland) Limited</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Ardintoul fish farm site</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>Yes, three farm technicians were on board the barge for lunch.</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>Moving slowly ahead</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>2018</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>Loch Alsh</t>
+        </is>
+      </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>Wind south-westerly at 15 knots, slight sea state, air temperature 5°C, water temperature about 7°C.</t>
+        </is>
+      </c>
+      <c r="P36" t="inlineStr">
+        <is>
+          <t>The crew member was transferred to the feed barge for lunch, then went to salmon cage 2 to remove dead fish.</t>
+        </is>
+      </c>
+      <c r="Q36" t="inlineStr">
+        <is>
+          <t>Lunch.</t>
+        </is>
+      </c>
+      <c r="R36" t="inlineStr">
+        <is>
+          <t>Polarcirkel rigid buoyancy boats (RBBs)</t>
+        </is>
+      </c>
+      <c r="S36" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T36" t="inlineStr">
+        <is>
+          <t>Yes, a "Mayday" call was made by the barge on VHF radio channel 16, and shortly afterwards a "Mayday" call from Beinn Na Caillich.  A fish farm technician also contacted the RBB crew by VHF radio.</t>
+        </is>
+      </c>
+      <c r="U36" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="V36" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="W36" t="inlineStr">
+        <is>
+          <t>No, Beinn Na Caillich’s crew had not conducted manoverboard drills and were unfamiliar with the workboat’s manoverboard recovery equipment. Emergency drills were rarely conducted.</t>
+        </is>
+      </c>
+      <c r="X36" t="inlineStr">
+        <is>
+          <t>1510</t>
+        </is>
+      </c>
+      <c r="Y36" t="inlineStr">
+        <is>
+          <t>5; Beinn Na Caillich's skipper, deckhand, Stolt Madah's skipper, and the three fish farm technicians</t>
+        </is>
+      </c>
+      <c r="Z36" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AA36" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AB36" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AC36" t="inlineStr">
+        <is>
+          <t>visibility good</t>
+        </is>
+      </c>
+      <c r="AD36" t="inlineStr">
+        <is>
+          <t>Yes, the vessel was moving slowly ahead.</t>
+        </is>
+      </c>
+      <c r="AE36" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AF36" t="inlineStr">
+        <is>
+          <t>570t</t>
+        </is>
+      </c>
+      <c r="AG36" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>2021-06-BeinnNaCaillich.pdf</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>gemini-1.5-flash-8b</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>1510</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Marine Harvest (Scotland) Limited</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Ardintoul fish farm site</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Yes, three farm technicians were on the barge for lunch.</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>Slowly ahead</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>2018</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>Loch Alsh</t>
+        </is>
+      </c>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>Wind south-westerly at 15 knots, slight sea state, air temperature 5°C, water temperature about 7°C.</t>
+        </is>
+      </c>
+      <c r="P37" t="inlineStr">
+        <is>
+          <t>The crew member, the assistant manager, was involved in transferring from a workboat to a barge.</t>
+        </is>
+      </c>
+      <c r="Q37" t="inlineStr">
+        <is>
+          <t>Lunch.</t>
+        </is>
+      </c>
+      <c r="R37" t="inlineStr">
+        <is>
+          <t>Polarcirkel rigid buoyancy boats (RBBs).</t>
+        </is>
+      </c>
+      <c r="S37" t="inlineStr">
+        <is>
+          <t>The technician grabbed hold of the strap at the back of the lifejacket.</t>
+        </is>
+      </c>
+      <c r="T37" t="inlineStr">
+        <is>
+          <t>Yes, Stornoway Coastguard received a "Mayday" call from the barge and shortly afterwards a "Mayday" call from Beinn Na Caillich.  A technician on the barge also contacted the RBB crew by VHF radio.</t>
+        </is>
+      </c>
+      <c r="U37" t="inlineStr">
+        <is>
+          <t>Not explicitly stated in the provided text.</t>
+        </is>
+      </c>
+      <c r="V37" t="inlineStr">
+        <is>
+          <t>Not applicable. The vessel was not carrying cargo.</t>
+        </is>
+      </c>
+      <c r="W37" t="inlineStr">
+        <is>
+          <t>No, Beinn Na Caillich’s crew had not conducted manoverboard drills and were unfamiliar with the workboat’s manoverboard recovery equipment.  Emergency drills were rarely conducted.</t>
+        </is>
+      </c>
+      <c r="X37" t="inlineStr">
+        <is>
+          <t>1510</t>
+        </is>
+      </c>
+      <c r="Y37" t="inlineStr">
+        <is>
+          <t>5; Beinn Na Caillich's skipper, deckhand, Stolt Madah's skipper, and the assistant manager and one technician on the barge.</t>
+        </is>
+      </c>
+      <c r="Z37" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AA37" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AB37" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AC37" t="inlineStr">
+        <is>
+          <t>visibility good</t>
+        </is>
+      </c>
+      <c r="AD37" t="inlineStr">
+        <is>
+          <t>yes, slowed to a slow speed ahead</t>
+        </is>
+      </c>
+      <c r="AE37" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AF37" t="inlineStr">
+        <is>
+          <t>570t</t>
+        </is>
+      </c>
+      <c r="AG37" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>2021-Seadogz_InterimReport.pdf</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>gemini-1.5-flash-8b</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>1011:09</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Seadogz Rib Charter Ltd</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Southampton Water</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>38.4kts (44.2mph)</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>2012</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>Southampton Water</t>
+        </is>
+      </c>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>Overcast with bright spells, winds 17kts from west-south-west with gusts of 25kts, slight sea state.</t>
+        </is>
+      </c>
+      <c r="P38" t="inlineStr">
+        <is>
+          <t>Concentrating on high-speed maneuvers in close proximity to another vessel, did not see the fixed navigational mark in time to take avoiding action.</t>
+        </is>
+      </c>
+      <c r="Q38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="U38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="V38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="W38" t="inlineStr">
+        <is>
+          <t>The skipper was a highly qualified and experienced RIB driver; he had local knowledge of Southampton Water and had worked for Seadogz Rib Charter Ltd on an ad-hoc basis for over 8 years.</t>
+        </is>
+      </c>
+      <c r="X38" t="inlineStr">
+        <is>
+          <t>1011:09</t>
+        </is>
+      </c>
+      <c r="Y38" t="inlineStr">
+        <is>
+          <t>12 passengers: two families of four, a party of two, and one individual passenger.</t>
+        </is>
+      </c>
+      <c r="Z38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AA38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AB38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AC38" t="inlineStr">
+        <is>
+          <t>good visibility</t>
+        </is>
+      </c>
+      <c r="AD38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AE38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AF38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AG38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>2021-Seadogz_InterimReport.pdf</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>gemini-1.5-flash-8b</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>1011:09</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Seadogz Rib Charter Ltd</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Southampton Water</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>38.4kts</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>2012</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>Southampton Water</t>
+        </is>
+      </c>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>Overcast with bright spells, winds 17kts from west-south-west with gusts of 25kts, slight sea state.</t>
+        </is>
+      </c>
+      <c r="P39" t="inlineStr">
+        <is>
+          <t>Concentrating on conducting high-speed manoeuvres in close proximity to another vessel and did not see the fixed navigational mark in time to take avoiding action.</t>
+        </is>
+      </c>
+      <c r="Q39" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R39" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S39" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T39" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="U39" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="V39" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="W39" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="X39" t="inlineStr">
+        <is>
+          <t>1011:09</t>
+        </is>
+      </c>
+      <c r="Y39" t="inlineStr">
+        <is>
+          <t>12 passengers, 2 crew, 10 injured, 1 fatality.</t>
+        </is>
+      </c>
+      <c r="Z39" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AA39" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AB39" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AC39" t="inlineStr">
+        <is>
+          <t>good visibility</t>
+        </is>
+      </c>
+      <c r="AD39" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AE39" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AF39" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AG39" t="inlineStr">
         <is>
           <t>-</t>
         </is>

</xml_diff>